<commit_message>
Improve scraping and data export handling
</commit_message>
<xml_diff>
--- a/data/opinions/188858911.xlsx
+++ b/data/opinions/188858911.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -819,12 +819,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>20357538</t>
+          <t>20404772</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>e...r</t>
+          <t>Adam</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -839,10 +839,14 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Wszystko w porządku</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>Bardzo dobra odsłona serii</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>fabuła, grafika, grywalność</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
@@ -856,24 +860,24 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-03-05 07:58:52</t>
+          <t>2026-03-24 07:53:28</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>2026-02-24 18:20:26</t>
+          <t>2026-03-20 12:35:37</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>20394775</t>
+          <t>20357538</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>m...4</t>
+          <t>e...r</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -888,7 +892,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Jest dobrze .</t>
+          <t>Wszystko w porządku</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -905,35 +909,39 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-03-19 16:04:15</t>
+          <t>2026-03-05 07:58:52</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>2026-02-26 05:15:25</t>
+          <t>2026-02-24 18:20:26</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>20345911</t>
+          <t>20394775</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>p bialczak</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>m...4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Polecam</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3/5</t>
+          <t>5/5</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Resident Evil Requiem zamówiony miesiąc przed premierą, nie dotarł do dzisiejszego dnia. Jak dotrze to zaktualizuje ocenę.</t>
+          <t>Jest dobrze .</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -945,17 +953,17 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-02-28 18:59:10</t>
+          <t>2026-03-19 16:04:15</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>2026-01-30 20:10:29</t>
+          <t>2026-02-26 05:15:25</t>
         </is>
       </c>
     </row>

</xml_diff>